<commit_message>
New CNN + GRU + DENSE -> XGBOOST Architecture. Mulitpliuer 1.1819 (+41.85%).
</commit_message>
<xml_diff>
--- a/models.xlsx
+++ b/models.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Dev\Trader_Artificial_Intelligence\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DF1C385-8B13-41CC-AD44-0CEAEA31CF59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA06E3A0-4CD2-435B-9A8F-ADD887960502}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="15">
   <si>
     <t>filename</t>
   </si>
@@ -78,6 +78,9 @@
   </si>
   <si>
     <t>Type de prédiction</t>
+  </si>
+  <si>
+    <t>hybridre_cnn_gru_dense_xgboost_return_1.4185</t>
   </si>
 </sst>
 </file>
@@ -121,9 +124,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -147,8 +151,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F994410D-5244-417F-B1AE-6C530DAB663A}" name="Table1" displayName="Table1" ref="A1:K3" totalsRowShown="0">
-  <autoFilter ref="A1:K3" xr:uid="{F994410D-5244-417F-B1AE-6C530DAB663A}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F994410D-5244-417F-B1AE-6C530DAB663A}" name="Table1" displayName="Table1" ref="A1:K4" totalsRowShown="0">
+  <autoFilter ref="A1:K4" xr:uid="{F994410D-5244-417F-B1AE-6C530DAB663A}"/>
   <tableColumns count="11">
     <tableColumn id="1" xr3:uid="{CA8ABE76-8A18-4FFF-90A7-D5F4889DE30D}" name="filename"/>
     <tableColumn id="11" xr3:uid="{8D1F8667-BF2F-4BC3-8DFD-58916E52D768}" name="Comet ML Name" dataCellStyle="Normal"/>
@@ -431,7 +435,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="56.140625" customWidth="1"/>
@@ -544,12 +548,47 @@
         <v>1.4711000000000001</v>
       </c>
       <c r="K3" s="1">
+        <v>0.18190000000000001</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4">
+        <v>0.1</v>
+      </c>
+      <c r="E4">
+        <v>0.1</v>
+      </c>
+      <c r="F4">
+        <v>0.84499999999999997</v>
+      </c>
+      <c r="G4">
+        <v>0.88</v>
+      </c>
+      <c r="H4">
+        <v>7.9000000000000001E-2</v>
+      </c>
+      <c r="I4">
+        <v>1.0999999999999999E-2</v>
+      </c>
+      <c r="J4">
+        <v>1.4185000000000001</v>
+      </c>
+      <c r="K4" s="1">
         <f>Table1[[#This Row],[Return]]-1</f>
-        <v>0.47110000000000007</v>
+        <v>0.41850000000000009</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="K1:K3 I4:I1048576">
+  <conditionalFormatting sqref="I5:I1048576 K1:K4">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -564,11 +603,12 @@
   <hyperlinks>
     <hyperlink ref="B2" r:id="rId1" display="https://www.comet.com/louisderveloy/trader-ai/a710d7d9c8964740b8d3020fd27f2223?&amp;prevPath=%2Flouisderveloy%2Ftrader-ai%2Fview%2Fnew%2Fpanels" xr:uid="{27059B99-9AAF-4BAE-A178-7FC4AB3FB99E}"/>
     <hyperlink ref="B3" r:id="rId2" display="https://www.comet.com/louisderveloy/trader-ai/a710d7d9c8964740b8d3020fd27f2223?&amp;prevPath=%2Flouisderveloy%2Ftrader-ai%2Fview%2Fnew%2Fpanels" xr:uid="{A3089BAE-BD9C-4E99-8483-89260B842C68}"/>
+    <hyperlink ref="B4" r:id="rId3" display="https://www.comet.com/louisderveloy/trader-ai/a710d7d9c8964740b8d3020fd27f2223?&amp;prevPath=%2Flouisderveloy%2Ftrader-ai%2Fview%2Fnew%2Fpanels" xr:uid="{E4D810E6-979F-4D01-B53A-D3FCC7EAC4C0}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId4"/>
   <tableParts count="1">
-    <tablePart r:id="rId4"/>
+    <tablePart r:id="rId5"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Added stat for better understanding of model performances
</commit_message>
<xml_diff>
--- a/models.xlsx
+++ b/models.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Dev\Trader_Artificial_Intelligence\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA06E3A0-4CD2-435B-9A8F-ADD887960502}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D362DBA9-C086-42D4-BE7C-B078BEAD5C85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1515" yWindow="1515" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -124,10 +124,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -558,7 +557,7 @@
       <c r="B4" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" t="s">
         <v>12</v>
       </c>
       <c r="D4">

</xml_diff>